<commit_message>
ios: frase fissa delle correzioni confermata da ChatGPT (EN, ES, FR, PT-BR, KO riviste)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ios/localizzazione/NEAT_novita.xlsx
+++ b/ios/localizzazione/NEAT_novita.xlsx
@@ -659,17 +659,17 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Bug fixes and small improvements.</t>
+          <t>Bug fixes and minor improvements.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Correcciones y pequeñas mejoras.</t>
+          <t>Corrección de errores y pequeñas mejoras.</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Corrections et petites améliorations.</t>
+          <t>Corrections de bugs et petites améliorations.</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Correções e pequenas melhorias.</t>
+          <t>Correções de bugs e pequenas melhorias.</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>버그 수정 및 작은 개선.</t>
+          <t>버그 수정 및 소소한 개선 사항.</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="P2" s="4" t="inlineStr">
         <is>
-          <t>Frase standard proposta da Claude (22 ottobre 2026), da confermare con ChatGPT nella chat delle traduzioni.</t>
+          <t>Frase standard confermata da ChatGPT il 22 ottobre 2026 (EN, ES, FR, PT-BR, KO riviste; DE, JA, ZH invariate).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ios 1.1: Novità, scheda dello store, privacy, supporto e note per il revisore con la copia in iCloud
Testi italiani approvati da Will il 26 ottobre 2026. Novità 1.1 nel foglio (traduzioni da fare), promozionale e
descrizione senza «nessun dato lascia il telefono», privacy e supporto in italiano e inglese, note per il revisore con
iCloud chiave-valore e Backup. Prompt per ChatGPT in localizzazione/PROMPT_CHATGPT_1.1.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ios/localizzazione/NEAT_novita.xlsx
+++ b/ios/localizzazione/NEAT_novita.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -631,15 +631,15 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="150" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>novita.correzioni</t>
+          <t>novita.1.1</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Novità (correzioni)</t>
+          <t>Novità 1.1</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -649,64 +649,108 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Testo fisso per le versioni di sola correzione (MAGGIORE.MINORE.CORREZIONE): nessuna funzione nuova da spiegare.</t>
+          <t>Versione 1.1. Copia automatica nel proprio iCloud (serie, obiettivi, impostazioni; mai i dati di Salute), backup manuale in un file dalle Impostazioni, promemoria serale corretto. Testo italiano approvato da Will il 26 ottobre 2026.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Correzioni e piccoli miglioramenti.</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Bug fixes and minor improvements.</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Corrección de errores y pequeñas mejoras.</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Corrections de bugs et petites améliorations.</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Fehlerbehebungen und kleine Verbesserungen.</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>Correções de bugs e pequenas melhorias.</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>不具合の修正と細かな改善。</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>버그 수정 및 소소한 개선 사항.</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>错误修复与小幅改进。</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>錯誤修正與小幅改進。</t>
-        </is>
-      </c>
+          <t>I tuoi progressi non si perdono più. Serie, obiettivi e impostazioni si salvano anche nel tuo iCloud: se cambi iPhone o reinstalli NEAT, ritrovi tutto, compresa la serie. Nulla però esce dal tuo account: i tuoi dati restano solo tuoi.
+• Nuovo in Impostazioni: «Backup». Salva i tuoi dati in un file e ricaricali quando vuoi.
+• Corretto il promemoria della sera: usa i passi più recenti e non arriva più se l'obiettivo è già raggiunto.
+• Piccole correzioni.</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="5" t="n"/>
+      <c r="J2" s="5" t="n"/>
+      <c r="K2" s="5" t="n"/>
+      <c r="L2" s="5" t="n"/>
+      <c r="M2" s="5" t="n"/>
+      <c r="N2" s="5" t="n"/>
       <c r="O2" s="4">
         <f>"EN: "&amp;LEN(F2)&amp;CHAR(10)&amp;"ES: "&amp;LEN(G2)&amp;CHAR(10)&amp;"FR: "&amp;LEN(H2)&amp;CHAR(10)&amp;"DE: "&amp;LEN(I2)&amp;CHAR(10)&amp;"PT-BR: "&amp;LEN(J2)&amp;CHAR(10)&amp;"JA: "&amp;LEN(K2)&amp;CHAR(10)&amp;"KO: "&amp;LEN(L2)&amp;CHAR(10)&amp;"ZH-Hans: "&amp;LEN(M2)&amp;CHAR(10)&amp;"ZH-Hant: "&amp;LEN(N2)</f>
         <v/>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>novita.correzioni</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Novità (correzioni)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>≤ 4000</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Testo fisso per le versioni di sola correzione (MAGGIORE.MINORE.CORREZIONE): nessuna funzione nuova da spiegare.</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Correzioni e piccoli miglioramenti.</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Bug fixes and minor improvements.</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Corrección de errores y pequeñas mejoras.</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Corrections de bugs et petites améliorations.</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Fehlerbehebungen und kleine Verbesserungen.</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Correções de bugs e pequenas melhorias.</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>不具合の修正と細かな改善。</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>버그 수정 및 소소한 개선 사항.</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>错误修复与小幅改进。</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>錯誤修正與小幅改進。</t>
+        </is>
+      </c>
+      <c r="O3" s="4">
+        <f>"EN: "&amp;LEN(F3)&amp;CHAR(10)&amp;"ES: "&amp;LEN(G3)&amp;CHAR(10)&amp;"FR: "&amp;LEN(H3)&amp;CHAR(10)&amp;"DE: "&amp;LEN(I3)&amp;CHAR(10)&amp;"PT-BR: "&amp;LEN(J3)&amp;CHAR(10)&amp;"JA: "&amp;LEN(K3)&amp;CHAR(10)&amp;"KO: "&amp;LEN(L3)&amp;CHAR(10)&amp;"ZH-Hans: "&amp;LEN(M3)&amp;CHAR(10)&amp;"ZH-Hant: "&amp;LEN(N3)</f>
+        <v/>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>Frase standard confermata da ChatGPT il 22 ottobre 2026 (EN, ES, FR, PT-BR, KO riviste; DE, JA, ZH invariate).</t>
         </is>

</xml_diff>

<commit_message>
ios 1.1: traduzioni di ChatGPT (Novità, scheda, screenshot 6, introduzione, Backup)
Fogli tornati da ChatGPT il 27 ottobre, controllati cella per cella: cambiate solo le righe richieste.
Tolti dal foglio i 7 testi dell'inserimento a mano, cataloghi e store/metadata.json rigenerati.
Didascalie dello screenshot 6 nel prompt per Claude Design.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ios/localizzazione/NEAT_novita.xlsx
+++ b/ios/localizzazione/NEAT_novita.xlsx
@@ -631,7 +631,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="150" customHeight="1">
+    <row r="2" ht="252" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
           <t>novita.1.1</t>
@@ -660,20 +660,95 @@
 • Piccole correzioni.</t>
         </is>
       </c>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
-      <c r="M2" s="5" t="n"/>
-      <c r="N2" s="5" t="n"/>
-      <c r="O2" s="4">
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You won't lose your progress anymore. Your streak, goals and settings are also saved in your iCloud: if you switch to another iPhone or reinstall NEAT, you get everything back, including your streak. Nothing leaves your Apple Account: your data is yours alone.
+• New in Settings: “Backup”. Save your data to a file and load it again whenever you want.
+• Fixed the evening reminder: it uses the latest step count and no longer arrives if you've already reached your goal.
+• Minor fixes.</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tus progresos ya no se pierden. Tu racha, tus objetivos y tus ajustes también se guardan en tu iCloud: si cambias de iPhone o reinstalas NEAT, lo recuperas todo, incluida tu racha. Nada sale de tu cuenta de Apple: tus datos siguen siendo solo tuyos.
+• Nuevo en Ajustes: «Copia de seguridad». Guarda tus datos en un archivo y vuelve a cargarlos cuando quieras.
+• Corregido el recordatorio nocturno: usa los pasos más recientes y ya no llega si has alcanzado tu objetivo.
+• Pequeñas correcciones.</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tes progrès ne se perdent plus. Ta série, tes objectifs et tes réglages sont aussi enregistrés dans ton iCloud : si tu changes d’iPhone ou réinstalles NEAT, tu retrouves tout, y compris ta série. Rien ne sort de ton compte Apple. Tes données, rien qu’à toi.
+• Nouveau dans Réglages : « Sauvegarde ». Enregistre tes données dans un fichier et recharge-les quand tu veux.
+• Le rappel du soir a été corrigé : il utilise les pas les plus récents et n’arrive plus si ton objectif est déjà atteint.
+• Petites corrections.</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deine Fortschritte gehen nicht mehr verloren. Deine Serie, Ziele und Einstellungen werden auch in deiner iCloud gesichert: Wenn du dein iPhone wechselst oder NEAT neu installierst, ist alles wieder da, auch deine Serie. Dabei verlässt nichts deinen Apple Account: Deine Daten gehören nur dir.
+• Neu in den Einstellungen: „Backup“. Speichere deine Daten in einer Datei und lade sie wieder, wann du willst.
+• Die Abenderinnerung wurde korrigiert: Sie nutzt die neuesten Schrittzahlen und kommt nicht mehr, wenn dein Ziel schon erreicht ist.
+• Kleine Fehlerbehebungen.</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seus progressos não se perdem mais. Sua sequência, metas e ajustes também são salvos no seu iCloud: se você trocar de iPhone ou reinstalar o NEAT, recupera tudo, inclusive sua sequência. Nada sai da sua Conta Apple: seus dados continuam sendo só seus.
+• Novo nos Ajustes: “Backup”. Salve seus dados em um arquivo e carregue-os de novo quando quiser.
+• O lembrete noturno foi corrigido: usa os passos mais recentes e não chega mais se você já atingiu sua meta.
+• Pequenas correções.</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">これまでの記録が失われなくなりました。連続記録、目標、設定があなたのiCloudにも保存されるようになりました。iPhoneを替えたりNEATを再インストールしたりしても、連続記録を含めてすべて元に戻ります。データがあなたのApple Accountの外に出ることはありません。あなたのデータは、あなただけのもの。
+• 設定に「バックアップ」を追加。データをファイルに保存して、いつでも読み込めます。
+• 夜のリマインダーを修正。最新の歩数を使い、目標を達成しているときは届かなくなりました。
+• 細かな不具合を修正。</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">이제 기록을 잃지 않아요. 연속 기록, 목표, 설정이 내 iCloud에도 저장돼요. iPhone을 바꾸거나 NEAT를 다시 설치해도 연속 기록을 포함해 모두 되찾을 수 있어요. 데이터는 내 Apple 계정 밖으로 나가지 않아요. 내 데이터는 나만의 것.
+• 설정에 ‘백업’이 생겼어요. 데이터를 파일로 저장하고 언제든 다시 불러올 수 있어요.
+• 저녁 알림을 수정했어요. 최신 걸음 수를 사용하고, 이미 목표를 달성했다면 더 이상 알림이 오지 않아요.
+• 사소한 오류를 수정했어요.</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">你的进度不会再丢失了。连续记录、目标和设置也会保存在你的iCloud中：更换iPhone或重新安装NEAT后，就能找回所有内容，包括连续记录。数据不会离开你的 Apple 账户，你的数据只属于你。
+• 设置中新增“备份”。将数据保存为文件，随时重新导入。
+• 修复了晚间提醒：使用最新步数，目标已达成时不再发送提醒。
+• 修复了一些小问题。</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">你的進度不會再遺失了。連續紀錄、目標和設定也會儲存在你的iCloud中：更換iPhone或重新安裝NEAT後，就能找回所有內容，包括連續紀錄。資料不會離開你的 Apple 帳號，你的資料只屬於你。
+• 設定中新增「備份」。將資料儲存為檔案，隨時重新匯入。
+• 修正了晚間提醒：使用最新步數，目標已達成時不再傳送提醒。
+• 修正了一些小問題。</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="str">
         <f>"EN: "&amp;LEN(F2)&amp;CHAR(10)&amp;"ES: "&amp;LEN(G2)&amp;CHAR(10)&amp;"FR: "&amp;LEN(H2)&amp;CHAR(10)&amp;"DE: "&amp;LEN(I2)&amp;CHAR(10)&amp;"PT-BR: "&amp;LEN(J2)&amp;CHAR(10)&amp;"JA: "&amp;LEN(K2)&amp;CHAR(10)&amp;"KO: "&amp;LEN(L2)&amp;CHAR(10)&amp;"ZH-Hans: "&amp;LEN(M2)&amp;CHAR(10)&amp;"ZH-Hant: "&amp;LEN(N2)</f>
-        <v/>
-      </c>
-      <c r="P2" s="4" t="n"/>
+        <v>EN: 486
+ES: 495
+FR: 516
+DE: 566
+PT-BR: 482
+JA: 260
+KO: 270
+ZH-Hans: 171
+ZH-Hant: 171</v>
+      </c>
+      <c r="P2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paragrafo iniziale e 3 punti conservati. Account Apple esplicitato; nome della sezione Backup coerente con le Impostazioni. JA/KO: progressi reso come registrazioni dell’app, nel contesto dei dati elencati. JA/KO/ZH: verifica madrelingua della privacy consigliata.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">

</xml_diff>